<commit_message>
chore: update ticket prices
</commit_message>
<xml_diff>
--- a/ticket_prices.xlsx
+++ b/ticket_prices.xlsx
@@ -18,6 +18,7 @@
     <sheet name="京都-水戸_822" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="町田-浦和_823" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="G大阪-広島_829" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="鹿島-G大阪_1009" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -8532,6 +8533,154 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>checked_at</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>エグゼクティブ・指定</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>カテゴリー１・指定</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>カテゴリー２・指定</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>カテゴリー３・指定</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>カテゴリー４・指定</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>カテゴリー５・指定</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>カテゴリー６・指定</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>ホームサポーターズシート・指定</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>ホームサポシコーナー・指定</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>ホームゴール裏北・指定</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>ビジター専用シート・指定</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>車椅子席</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-09-30 06:01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>9,600 完売</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>7,000</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>6,000</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>6,400</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>5,400</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>5,100</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>4,900</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>3,700</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>4,000</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>4,000</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>3,700</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>3,700</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>